<commit_message>
Login com sucesso OK
</commit_message>
<xml_diff>
--- a/src/test/resources/dados/MassaDados.xlsx
+++ b/src/test/resources/dados/MassaDados.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DEV\TREINAMENTO\src\test\resources\dados\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\myGithub\javaMobileAppiumTests\src\test\resources\dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84D76439-CC9C-46F5-84F3-D5FA12FD50D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDB5C55E-2D61-448B-9643-1957C93D0AF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2295" yWindow="45" windowWidth="17715" windowHeight="10740" xr2:uid="{BE8CC490-7143-461B-A081-5E1B4D404489}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="22245" windowHeight="15585" xr2:uid="{BE8CC490-7143-461B-A081-5E1B4D404489}"/>
   </bookViews>
   <sheets>
-    <sheet name="USUARIO" sheetId="1" r:id="rId1"/>
-    <sheet name="USUARIO_SECUNDARIO" sheetId="2" r:id="rId2"/>
+    <sheet name="EBAC_MASSAS" sheetId="3" r:id="rId1"/>
+    <sheet name="USUARIO" sheetId="1" r:id="rId2"/>
+    <sheet name="USUARIO_SECUNDARIO" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="60">
   <si>
     <t>TAG</t>
   </si>
@@ -178,13 +179,52 @@
   </si>
   <si>
     <t>78046552313</t>
+  </si>
+  <si>
+    <t>FIRST NAME</t>
+  </si>
+  <si>
+    <t>LAST NAME</t>
+  </si>
+  <si>
+    <t>PHONE</t>
+  </si>
+  <si>
+    <t>EMAIL</t>
+  </si>
+  <si>
+    <t>PASSWORD</t>
+  </si>
+  <si>
+    <t>CT-1007</t>
+  </si>
+  <si>
+    <t>CT-1008</t>
+  </si>
+  <si>
+    <t>CT-1009</t>
+  </si>
+  <si>
+    <t>CT-1010</t>
+  </si>
+  <si>
+    <t>emmy.herman@miller.biz</t>
+  </si>
+  <si>
+    <t>&gt;ocb"8QN)C$=sIa"]Kp</t>
+  </si>
+  <si>
+    <t>elva.torphy@yahoo.com</t>
+  </si>
+  <si>
+    <t>VR%RzRqQRxD[.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -202,6 +242,20 @@
       <u/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10.5"/>
+      <color rgb="FF98C379"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -224,10 +278,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -256,8 +311,13 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -589,9 +649,116 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AF78ECA-9F9C-408E-8B71-24EBCB9A0622}">
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="4" max="6" width="8.85546875" customWidth="1"/>
+    <col min="7" max="7" width="28.5703125" customWidth="1"/>
+    <col min="8" max="8" width="21.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G1" t="s">
+        <v>50</v>
+      </c>
+      <c r="H1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="H3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" t="s">
+        <v>55</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="G3" r:id="rId1" xr:uid="{B0308FEC-1770-4F1D-BB0B-F48CC96B8527}"/>
+  </hyperlinks>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3A74B6D-8FA4-4011-9C72-01FBA93CFAED}">
   <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.28515625" style="2" bestFit="1" customWidth="1"/>
@@ -601,7 +768,7 @@
     <col min="8" max="8" width="21.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -627,7 +794,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8">
       <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
@@ -653,7 +820,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8">
       <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
@@ -679,7 +846,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8">
       <c r="A4" s="2" t="s">
         <v>8</v>
       </c>
@@ -705,7 +872,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8">
       <c r="A5" s="2" t="s">
         <v>9</v>
       </c>
@@ -731,7 +898,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8">
       <c r="A6" s="2" t="s">
         <v>12</v>
       </c>
@@ -757,7 +924,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8">
       <c r="A7" s="2" t="s">
         <v>11</v>
       </c>
@@ -783,7 +950,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8">
       <c r="A8" s="2" t="s">
         <v>19</v>
       </c>
@@ -809,7 +976,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8">
       <c r="A9" s="2" t="s">
         <v>37</v>
       </c>
@@ -835,7 +1002,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8">
       <c r="A10" s="2" t="s">
         <v>39</v>
       </c>
@@ -861,7 +1028,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8">
       <c r="A11" s="2" t="s">
         <v>43</v>
       </c>
@@ -894,12 +1061,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D587F36B-31B9-45A1-B9D4-E7990020F21E}">
   <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -922,7 +1089,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7">
       <c r="A2" s="2" t="s">
         <v>43</v>
       </c>

</xml_diff>

<commit_message>
Refactor passagens steps and actions for flight selection
Updated PassagensActions and PassagensSteps to clarify and separate the selection of outbound and return flights. Step definitions and feature file steps were renamed for better readability and alignment with user actions. Also updated data selection logic to use return date and added new methods for selecting and confirming return flights.
</commit_message>
<xml_diff>
--- a/src/test/resources/dados/MassaDados.xlsx
+++ b/src/test/resources/dados/MassaDados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DEV\AUTOMACAO\javaMobileAppiumTests\src\test\resources\dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F4301DA-879E-4307-A331-6F873690A6CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4719EB6-234E-463A-BB87-7C2D6457CC87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="25065" yWindow="45" windowWidth="16020" windowHeight="10905" xr2:uid="{BE8CC490-7143-461B-A081-5E1B4D404489}"/>
   </bookViews>
@@ -716,15 +716,15 @@
       </c>
       <c r="I4" s="1" t="str">
         <f t="shared" ref="I4" ca="1" si="3">DAY(M4) &amp; ""</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L4" s="11">
-        <f ca="1">TODAY()+5</f>
+        <f ca="1">TODAY()+ 5</f>
         <v>45838</v>
       </c>
       <c r="M4" s="11">
-        <f ca="1">TODAY()+21</f>
-        <v>45854</v>
+        <f ca="1">TODAY()+22</f>
+        <v>45855</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">

</xml_diff>